<commit_message>
update: sync seating and guest changes from google sheets
</commit_message>
<xml_diff>
--- a/data/filled_from_gsheet.xlsx
+++ b/data/filled_from_gsheet.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J87"/>
+  <dimension ref="A2:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>林浩生</t>
+          <t>林素霞</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>女方-舅公</t>
+          <t>女方-姨婆</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>林素霞</t>
+          <t>林春霞</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>林春霞</t>
+          <t>林麗霞</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1972,17 +1972,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>林麗霞</t>
+          <t>吳慧儀</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>天外奇蹟</t>
+          <t>小美人魚</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>女方-姨婆</t>
+          <t>女方-姨丈的姊姊</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>吳慧儀</t>
+          <t>吳宗鴻</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>女方-姨丈的姊姊</t>
+          <t>女方-姨丈</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>吳宗鴻</t>
+          <t>郭乃萍</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2038,16 +2038,18 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>女方-姨丈</t>
+          <t>女方-阿姨</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>中西式</t>
-        </is>
-      </c>
-      <c r="H55" t="n">
-        <v>8</v>
+          <t>其他代表領取</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>好命婆</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -2056,7 +2058,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>郭乃萍</t>
+          <t>吳誼萱</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2066,17 +2068,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>女方-阿姨</t>
+          <t>女方-表妹</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>其他代表領取</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>好命婆</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2083,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>吳誼萱</t>
+          <t>吳瑞臻</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2111,7 +2108,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>吳瑞臻</t>
+          <t>吳芷瑋</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2136,23 +2133,26 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>吳芷瑋</t>
+          <t>羅秋香</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>小美人魚</t>
+          <t>美女與野獸</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>女方-表妹</t>
+          <t>男方-姑姑</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>其他代表領取</t>
-        </is>
+          <t>已領取</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="60">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>羅秋香</t>
+          <t>羅秀琴</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>羅秀琴</t>
+          <t>羅冬燮</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>男方-姑姑</t>
+          <t>男方-堂伯父</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>羅冬燮</t>
+          <t>羅家豐</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>羅家豐</t>
+          <t>羅時逢</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>男方-堂伯父</t>
+          <t>男方-司機叔叔</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>羅時逢</t>
+          <t>羅聖評</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>美女與野獸</t>
+          <t>仙履奇緣</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>男方-司機叔叔</t>
+          <t>男方-哥哥</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>羅聖評</t>
+          <t>羅婕寧</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>男方-哥哥</t>
+          <t>男方-姊姊</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>羅婕寧</t>
+          <t>張峻維</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>男方-姊姊</t>
+          <t>男方-親戚</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>張峻維</t>
+          <t>張峻源</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>張峻源</t>
+          <t>張峻愷</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>張峻愷</t>
+          <t>張育綾</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>張育綾</t>
+          <t>張育真</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>張育真</t>
+          <t>陳宏益</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>陳宏益</t>
+          <t>陳思語</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2525,17 +2525,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>陳思語</t>
+          <t>張敏珠</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>仙履奇緣</t>
+          <t>變身國王</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>男方-親戚</t>
+          <t>男方-阿姨</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>張敏珠</t>
+          <t>陳銘鳳</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>男方-阿姨</t>
+          <t>男方-姨丈</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>陳銘鳳</t>
+          <t>陳中佑</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>男方-姨丈</t>
+          <t>男方-親戚</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>陳中佑</t>
+          <t>陳麗絲</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>陳麗絲</t>
+          <t>張添吉</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>男方-親戚</t>
+          <t>男方-舅舅</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>張添吉</t>
+          <t>黃彩朋</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>男方-舅舅</t>
+          <t>男方-舅媽</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>黃彩朋</t>
+          <t>張睿善</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>男方-舅媽</t>
+          <t>男方-表弟</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>張睿善</t>
+          <t>張雅茹</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>男方-表弟</t>
+          <t>男方-表妹</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>張雅茹</t>
+          <t>姜義璽</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>男方-表妹</t>
+          <t>男方-表妹夫</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>姜義璽</t>
+          <t>姜禮豪</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>男方-表妹夫</t>
+          <t>男方-表姪</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2805,22 +2805,22 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>姜禮豪</t>
+          <t>郭乃瑜</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>變身國王</t>
+          <t>睡美人</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>男方-表姪</t>
+          <t>女方-阿姨</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>已領取</t>
+          <t>中西式</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>郭乃瑜</t>
+          <t>郭祐任</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>女方-阿姨</t>
+          <t>女方-舅舅</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>郭祐任</t>
+          <t>張雅嵐</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2871,16 +2871,13 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>女方-舅舅</t>
+          <t>女方-舅媽</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
           <t>中西式</t>
         </is>
-      </c>
-      <c r="H85" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="86">
@@ -2889,7 +2886,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>張雅嵐</t>
+          <t>郭丁綺</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2899,38 +2896,10 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>女方-舅媽</t>
+          <t>女方-表妹</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
-        <is>
-          <t>中西式</t>
-        </is>
-      </c>
-      <c r="H86" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n">
-        <v>84</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>郭丁綺</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>睡美人</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>女方-表妹</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
         <is>
           <t>其他代表領取</t>
         </is>
@@ -3364,12 +3333,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>林浩生</t>
+          <t>林素霞</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>女方舅公</t>
+          <t>女方姨婆</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3348,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>林浩生親戚</t>
+          <t>林素霞親戚</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3373,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>林素霞親戚</t>
+          <t>林素霞媳婦</t>
         </is>
       </c>
     </row>
@@ -3412,14 +3381,9 @@
       <c r="A39" t="n">
         <v>7</v>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>林春霞</t>
-        </is>
-      </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>女方姨婆</t>
+          <t>林素霞孫子</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3393,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>林春霞親戚</t>
+          <t>林素霞孫子</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: sync latest seating and guest list from Google Sheet (added 江仁杉, 陳威銘 to 金銀島)
</commit_message>
<xml_diff>
--- a/data/filled_from_gsheet.xlsx
+++ b/data/filled_from_gsheet.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J86"/>
+  <dimension ref="A2:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -1489,31 +1489,26 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>立苓/LiLing</t>
+          <t>江仁杉</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>冰雪奇緣</t>
+          <t>金銀島</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>女方-朋友</t>
+          <t>男生-朋友</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>西式</t>
+          <t>中式</t>
         </is>
       </c>
       <c r="H37" t="n">
         <v>1</v>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>0970502332</t>
-        </is>
       </c>
     </row>
     <row r="38">
@@ -1522,31 +1517,26 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>周琬玲</t>
+          <t>陳威銘</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>冰雪奇緣</t>
+          <t>金銀島</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>女方-朋友</t>
+          <t>男生-朋友</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>西式</t>
+          <t>中式</t>
         </is>
       </c>
       <c r="H38" t="n">
         <v>1</v>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>0970581016</t>
-        </is>
       </c>
     </row>
     <row r="39">
@@ -1555,7 +1545,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>楊雅筑</t>
+          <t>立苓/LiLing</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1578,7 +1568,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>0912397067</t>
+          <t>0970502332</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1578,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>楊亞霖</t>
+          <t>周琬玲</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1607,11 +1597,11 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>0970987715</t>
+          <t>0970581016</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1611,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>楊建成</t>
+          <t>楊雅筑</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1644,7 +1634,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>0973970178</t>
+          <t>0912397067</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1644,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>張晉瑋</t>
+          <t>楊亞霖</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1673,11 +1663,11 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>0918747233</t>
+          <t>0970987715</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1677,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>謝坤森</t>
+          <t>楊建成</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1710,7 +1700,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>0955760556</t>
+          <t>0973970178</t>
         </is>
       </c>
     </row>
@@ -1720,17 +1710,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>施定仁</t>
+          <t>張晉瑋</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>熊的傳說</t>
+          <t>冰雪奇緣</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>女方-家長朋友</t>
+          <t>女方-朋友</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1739,7 +1729,12 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>0918747233</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1748,17 +1743,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>江明陽</t>
+          <t>謝坤森</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>熊的傳說</t>
+          <t>冰雪奇緣</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>女方-家長朋友</t>
+          <t>女方-朋友</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1767,7 +1762,12 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>0955760556</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>許明炳</t>
+          <t>施定仁</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>鄭淙銘</t>
+          <t>江明陽</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>高凰文</t>
+          <t>許明炳</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1860,22 +1860,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>林燦生</t>
+          <t>鄭淙銘</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>天外奇蹟</t>
+          <t>熊的傳說</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>女方-舅公</t>
+          <t>女方-家長朋友</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>中西式</t>
+          <t>西式</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -1888,22 +1888,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>林素霞</t>
+          <t>高凰文</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>天外奇蹟</t>
+          <t>熊的傳說</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>女方-姨婆</t>
+          <t>女方-家長朋友</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>中西式</t>
+          <t>西式</t>
         </is>
       </c>
       <c r="H50" t="n">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>林春霞</t>
+          <t>林燦生</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>女方-姨婆</t>
+          <t>女方-舅公</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>林麗霞</t>
+          <t>林素霞</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1972,17 +1972,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>吳慧儀</t>
+          <t>林春霞</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>小美人魚</t>
+          <t>天外奇蹟</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>女方-姨丈的姊姊</t>
+          <t>女方-姨婆</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54">
@@ -2000,17 +2000,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>吳宗鴻</t>
+          <t>林麗霞</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>小美人魚</t>
+          <t>天外奇蹟</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>女方-姨丈</t>
+          <t>女方-姨婆</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>郭乃萍</t>
+          <t>吳慧儀</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2038,18 +2038,16 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>女方-阿姨</t>
+          <t>女方-姨丈的姊姊</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>其他代表領取</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>好命婆</t>
-        </is>
+          <t>中西式</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="56">
@@ -2058,7 +2056,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>吳誼萱</t>
+          <t>吳宗鴻</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2068,13 +2066,16 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>女方-表妹</t>
+          <t>女方-姨丈</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>其他代表領取</t>
-        </is>
+          <t>中西式</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="57">
@@ -2083,7 +2084,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>吳瑞臻</t>
+          <t>郭乃萍</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2093,12 +2094,17 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>女方-表妹</t>
+          <t>女方-阿姨</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
           <t>其他代表領取</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>好命婆</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2114,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>吳芷瑋</t>
+          <t>吳誼萱</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2133,26 +2139,23 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>羅秋香</t>
+          <t>吳瑞臻</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>美女與野獸</t>
+          <t>小美人魚</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>男方-姑姑</t>
+          <t>女方-表妹</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>已領取</t>
-        </is>
-      </c>
-      <c r="H59" t="n">
-        <v>2</v>
+          <t>其他代表領取</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -2161,26 +2164,23 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>羅秀琴</t>
+          <t>吳芷瑋</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>美女與野獸</t>
+          <t>小美人魚</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>男方-姑姑</t>
+          <t>女方-表妹</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>已領取</t>
-        </is>
-      </c>
-      <c r="H60" t="n">
-        <v>2</v>
+          <t>其他代表領取</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>羅冬燮</t>
+          <t>羅秋香</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>男方-堂伯父</t>
+          <t>男方-姑姑</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>羅家豐</t>
+          <t>羅秀琴</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>男方-堂伯父</t>
+          <t>男方-姑姑</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>羅時逢</t>
+          <t>羅冬燮</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>男方-司機叔叔</t>
+          <t>男方-堂伯父</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>羅聖評</t>
+          <t>羅家豐</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>仙履奇緣</t>
+          <t>美女與野獸</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>男方-哥哥</t>
+          <t>男方-堂伯父</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
@@ -2301,17 +2301,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>羅婕寧</t>
+          <t>羅時逢</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>仙履奇緣</t>
+          <t>美女與野獸</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>男方-姊姊</t>
+          <t>男方-司機叔叔</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>張峻維</t>
+          <t>羅聖評</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>男方-親戚</t>
+          <t>男方-哥哥</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>張峻源</t>
+          <t>羅婕寧</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>男方-親戚</t>
+          <t>男方-姊姊</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>張峻愷</t>
+          <t>張峻維</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>張育綾</t>
+          <t>張峻源</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>張育真</t>
+          <t>張峻愷</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>陳宏益</t>
+          <t>張育綾</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>陳思語</t>
+          <t>張育真</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2525,17 +2525,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>張敏珠</t>
+          <t>陳宏益</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>變身國王</t>
+          <t>仙履奇緣</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>男方-阿姨</t>
+          <t>男方-親戚</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2553,17 +2553,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>陳銘鳳</t>
+          <t>陳思語</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>變身國王</t>
+          <t>仙履奇緣</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>男方-姨丈</t>
+          <t>男方-親戚</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>陳中佑</t>
+          <t>張敏珠</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>男方-親戚</t>
+          <t>男方-阿姨</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>陳麗絲</t>
+          <t>陳銘鳳</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>男方-親戚</t>
+          <t>男方-姨丈</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>張添吉</t>
+          <t>陳中佑</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>男方-舅舅</t>
+          <t>男方-親戚</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>黃彩朋</t>
+          <t>陳麗絲</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>男方-舅媽</t>
+          <t>男方-親戚</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>張睿善</t>
+          <t>張添吉</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>男方-表弟</t>
+          <t>男方-舅舅</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>張雅茹</t>
+          <t>黃彩朋</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>男方-表妹</t>
+          <t>男方-舅媽</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>姜義璽</t>
+          <t>張睿善</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>男方-表妹夫</t>
+          <t>男方-表弟</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>姜禮豪</t>
+          <t>張雅茹</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>男方-表姪</t>
+          <t>男方-表妹</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2805,22 +2805,22 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>郭乃瑜</t>
+          <t>姜義璽</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>睡美人</t>
+          <t>變身國王</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>女方-阿姨</t>
+          <t>男方-表妹夫</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>中西式</t>
+          <t>已領取</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -2833,26 +2833,26 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>郭祐任</t>
+          <t>姜禮豪</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>睡美人</t>
+          <t>變身國王</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>女方-舅舅</t>
+          <t>男方-表姪</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>中西式</t>
+          <t>已領取</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>張雅嵐</t>
+          <t>郭乃瑜</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2871,13 +2871,16 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>女方-舅媽</t>
+          <t>女方-阿姨</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
           <t>中西式</t>
         </is>
+      </c>
+      <c r="H85" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -2886,20 +2889,73 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
+          <t>郭祐任</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>睡美人</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>女方-舅舅</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>中西式</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>84</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>張雅嵐</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>睡美人</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>女方-舅媽</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>中西式</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>85</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>郭丁綺</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>睡美人</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>女方-表妹</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G88" t="inlineStr">
         <is>
           <t>其他代表領取</t>
         </is>
@@ -4211,11 +4267,31 @@
       <c r="A110" t="n">
         <v>8</v>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>江仁杉</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>男方朋友</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
         <v>9</v>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>陳威銘</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>男方朋友</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4225,7 +4301,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">　本桌（總表已分配）：7 人</t>
+          <t xml:space="preserve">　本桌（總表已分配）：9 人</t>
         </is>
       </c>
     </row>

</xml_diff>